<commit_message>
chore: align bulk order download template
</commit_message>
<xml_diff>
--- a/public/templates/jeongilpum-bulk-orders.xlsx
+++ b/public/templates/jeongilpum-bulk-orders.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="주문입력" sheetId="1" r:id="Re4c628fc7b434248"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성안내" sheetId="2" r:id="R6e2aac307b1f43d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상품코드표" sheetId="3" r:id="R94fcd61931474163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="주문입력" sheetId="1" r:id="R0c0f34d05f094415"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성안내" sheetId="2" r:id="Ra4ccc51b170b412f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상품코드표" sheetId="3" r:id="R1002be3016e14a25"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5687,7 +5687,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc385893e007f4ee2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11641fe64cf94c21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13086,7 +13086,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30a521190f404315"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re594dd00fc604566"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>